<commit_message>
Stage 3.5: three datasets, WEDA-trained motion model
</commit_message>
<xml_diff>
--- a/eval/outputs/Motion_Model_Selection.xlsx
+++ b/eval/outputs/Motion_Model_Selection.xlsx
@@ -11,6 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First run (6 models)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FallAllD" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final test" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Three datasets" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,9 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="+0.000;-0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -90,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,6 +133,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2032,4 +2045,817 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Final XGBoost model, one-time test (impact segments that pass the 2.25 g gate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Test set</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Falls</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ADLs</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AUC (XGBoost)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>AUC (gate only)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Falls caught at 0.926</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>False alarms / hour at 0.926</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall test subjects (S02, S06, S11)</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>FallAllD report half (S01, S02, S03, S09, S12, S13)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>271</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>966</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>0.498</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Full stream, one score per recording (AUC / falls caught at 95% specificity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Test set</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Recordings</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Fall recordings</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Impact only: AUC</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Impact only: caught</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Impact + stillness: AUC</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Impact + stillness: caught</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall test subjects</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>0.944</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>FallAllD report half</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>1237</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>271</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>0.365</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Model trained on 15 UMAFall subjects only. Threshold 0.926 set on those subjects (95% specificity).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Run once; the test data were not used for any choice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>UMAFall test is 3 people with staged falls onto a mattress. FallAllD report half is the cross-dataset result.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dev parts: train on one or two datasets, score on all three (gated AUC; own data = leave-one-person-out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Trained on</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Setting (depth, trees, lambda)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>UMAFall</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FallAllD</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>WEDA-FALL</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Mean on unseen datasets</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>WEDA faint-type falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>2, 50, 10</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>0.983</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>0.654</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>0.748</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>FallAllD</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>2, 100, 1</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0.588</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>WEDA-FALL (winner)</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>4, 100, 1</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall + FallAllD</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>2, 50, 1</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0.673</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0.761</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall + WEDA-FALL</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>2, 300, 1</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>FallAllD + WEDA-FALL</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>2, 100, 10</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>One-time test on the locked test parts (alarm = gate fired and score at or above the threshold)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Test set</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Seen in training?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Falls</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ADLs</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>AUC (gated)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Falls caught</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>False alarms / hour</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Faint-type caught</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Elderly ADL false alarms</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>WEDA-trained (winner), threshold 0.886</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>UMAFall (S02, S06, S11)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Unseen dataset</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>WEDA-trained (winner), threshold 0.886</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>FallAllD report half</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Unseen dataset</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>271</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>966</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>WEDA-trained (winner), threshold 0.886</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>WEDA-FALL (U04, U07, U08, U10, U21, U22, U29)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>New people</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>0 of 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall-trained (old), threshold 0.926</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>UMAFall (S02, S06, S11)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>New people</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall-trained (old), threshold 0.926</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>FallAllD report half</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Unseen dataset</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>271</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>966</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0.498</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>UMAFall-trained (old), threshold 0.926</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>WEDA-FALL (U04, U07, U08, U10, U21, U22, U29)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Unseen dataset</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>0.795</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>1 of 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Same signal path for all three: clip at 8 g, 20 Hz, 2.25 g gate, 18 features, XGBoost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Rule used: drop the 0.95 own-data floor (only UMAFall could reach it). Pooling beat both single datasets on 1 of 3 unseen datasets, so the best single dataset wins: WEDA-FALL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Test run once; the winner was fixed before it. Mean on unseen datasets: winner 0.792, old model 0.745. On FallAllD, unseen by both, they are level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Thresholds set on one dataset do not carry over: the winner misses falls on other data, the old model raises many false alarms. The real band needs its own threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Saved as models/motion.joblib (697 WEDA-FALL dev segments, 250 falls). Old model kept as models/motion_umafall_stage3.joblib.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Stage 3.5b: full WEDA tuning, kept current model
</commit_message>
<xml_diff>
--- a/eval/outputs/Motion_Model_Selection.xlsx
+++ b/eval/outputs/Motion_Model_Selection.xlsx
@@ -2286,7 +2286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2855,6 +2855,13 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Full tuning of the WEDA model afterwards (258 settings, dev only): best was 0.810 on unseen datasets vs 0.809 for the current setting. Below the 0.01 needed to switch, so the model was kept.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>